<commit_message>
Soprannomi da pagine Wikipedia con cache, varianti del nome; docs aggiornate
</commit_message>
<xml_diff>
--- a/output/asta.xlsx
+++ b/output/asta.xlsx
@@ -42913,7 +42913,11 @@
         </is>
       </c>
       <c r="C333" s="3" t="inlineStr"/>
-      <c r="D333" s="3" t="inlineStr"/>
+      <c r="D333" s="3" t="inlineStr">
+        <is>
+          <t>Ché Zach Everton Fred Adams</t>
+        </is>
+      </c>
       <c r="E333" s="3" t="inlineStr">
         <is>
           <t>A</t>
@@ -43063,7 +43067,11 @@
         </is>
       </c>
       <c r="C334" t="inlineStr"/>
-      <c r="D334" t="inlineStr"/>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Akor Jerome Adams</t>
+        </is>
+      </c>
       <c r="E334" t="inlineStr">
         <is>
           <t>A</t>
@@ -43285,7 +43293,11 @@
         </is>
       </c>
       <c r="C336" t="inlineStr"/>
-      <c r="D336" t="inlineStr"/>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Albion Rrahmani</t>
+        </is>
+      </c>
       <c r="E336" t="inlineStr">
         <is>
           <t>A</t>
@@ -43391,7 +43403,11 @@
         </is>
       </c>
       <c r="C337" t="inlineStr"/>
-      <c r="D337" t="inlineStr"/>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Pontus Skule Erik Almqvist</t>
+        </is>
+      </c>
       <c r="E337" t="inlineStr">
         <is>
           <t>A</t>
@@ -43655,7 +43671,11 @@
         </is>
       </c>
       <c r="C339" t="inlineStr"/>
-      <c r="D339" t="inlineStr"/>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Domenico Berardi</t>
+        </is>
+      </c>
       <c r="E339" t="inlineStr">
         <is>
           <t>A</t>
@@ -43791,7 +43811,11 @@
         </is>
       </c>
       <c r="C340" t="inlineStr"/>
-      <c r="D340" t="inlineStr"/>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Norberto Bercique Gomes Betuncal</t>
+        </is>
+      </c>
       <c r="E340" t="inlineStr">
         <is>
           <t>A</t>
@@ -43899,7 +43923,11 @@
         </is>
       </c>
       <c r="C341" t="inlineStr"/>
-      <c r="D341" t="inlineStr"/>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>George Daniel Bîrligea</t>
+        </is>
+      </c>
       <c r="E341" t="inlineStr">
         <is>
           <t>A</t>
@@ -44005,7 +44033,11 @@
         </is>
       </c>
       <c r="C342" t="inlineStr"/>
-      <c r="D342" t="inlineStr"/>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Tomáš Bobček</t>
+        </is>
+      </c>
       <c r="E342" t="inlineStr">
         <is>
           <t>A</t>
@@ -44111,7 +44143,11 @@
         </is>
       </c>
       <c r="C343" s="3" t="inlineStr"/>
-      <c r="D343" s="3" t="inlineStr"/>
+      <c r="D343" s="3" t="inlineStr">
+        <is>
+          <t>Jérémie Boga</t>
+        </is>
+      </c>
       <c r="E343" s="3" t="inlineStr">
         <is>
           <t>A</t>
@@ -44261,7 +44297,11 @@
         </is>
       </c>
       <c r="C344" t="inlineStr"/>
-      <c r="D344" t="inlineStr"/>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Ange-Yoan Laurent Bonny</t>
+        </is>
+      </c>
       <c r="E344" t="inlineStr">
         <is>
           <t>A</t>
@@ -44393,7 +44433,11 @@
         </is>
       </c>
       <c r="C345" t="inlineStr"/>
-      <c r="D345" t="inlineStr"/>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Kieron Thomas Bowie</t>
+        </is>
+      </c>
       <c r="E345" t="inlineStr">
         <is>
           <t>A</t>
@@ -44797,7 +44841,11 @@
         </is>
       </c>
       <c r="C348" t="inlineStr"/>
-      <c r="D348" t="inlineStr"/>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Matteo Cancellieri</t>
+        </is>
+      </c>
       <c r="E348" t="inlineStr">
         <is>
           <t>A</t>
@@ -45200,8 +45248,16 @@
           <t>Cutrone</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr"/>
-      <c r="D351" t="inlineStr"/>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Pokémon</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Patrick Cutrone</t>
+        </is>
+      </c>
       <c r="E351" t="inlineStr">
         <is>
           <t>A</t>
@@ -45307,7 +45363,11 @@
         </is>
       </c>
       <c r="C352" t="inlineStr"/>
-      <c r="D352" t="inlineStr"/>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Dany Mota Carvalho</t>
+        </is>
+      </c>
       <c r="E352" t="inlineStr">
         <is>
           <t>A</t>
@@ -45545,7 +45605,11 @@
         </is>
       </c>
       <c r="C354" t="inlineStr"/>
-      <c r="D354" t="inlineStr"/>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Keinan Vincent Joseph Davis</t>
+        </is>
+      </c>
       <c r="E354" t="inlineStr">
         <is>
           <t>A</t>
@@ -45681,7 +45745,11 @@
         </is>
       </c>
       <c r="C355" t="inlineStr"/>
-      <c r="D355" t="inlineStr"/>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Charles Marc De Ketelaere</t>
+        </is>
+      </c>
       <c r="E355" t="inlineStr">
         <is>
           <t>A</t>
@@ -45817,7 +45885,11 @@
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr"/>
-      <c r="D356" s="2" t="inlineStr"/>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>Assane Diao Diaoune</t>
+        </is>
+      </c>
       <c r="E356" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -46085,7 +46157,11 @@
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr"/>
-      <c r="D358" s="2" t="inlineStr"/>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>Anastasios Douvikas</t>
+        </is>
+      </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -46221,7 +46297,11 @@
         </is>
       </c>
       <c r="C359" s="3" t="inlineStr"/>
-      <c r="D359" s="3" t="inlineStr"/>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>Artem Dovbyk</t>
+        </is>
+      </c>
       <c r="E359" s="3" t="inlineStr">
         <is>
           <t>A</t>
@@ -46370,8 +46450,16 @@
           <t>Dybala</t>
         </is>
       </c>
-      <c r="C360" s="2" t="inlineStr"/>
-      <c r="D360" s="2" t="inlineStr"/>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>la Joya</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>Paulo Exequiel Dybala</t>
+        </is>
+      </c>
       <c r="E360" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -46863,7 +46951,11 @@
         </is>
       </c>
       <c r="C364" t="inlineStr"/>
-      <c r="D364" t="inlineStr"/>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Sebastiano Esposito</t>
+        </is>
+      </c>
       <c r="E364" t="inlineStr">
         <is>
           <t>A</t>
@@ -46995,7 +47087,11 @@
         </is>
       </c>
       <c r="C365" t="inlineStr"/>
-      <c r="D365" t="inlineStr"/>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Francesco Pio Esposito</t>
+        </is>
+      </c>
       <c r="E365" t="inlineStr">
         <is>
           <t>A</t>
@@ -47387,7 +47483,11 @@
         </is>
       </c>
       <c r="C368" t="inlineStr"/>
-      <c r="D368" t="inlineStr"/>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Seydou Fini</t>
+        </is>
+      </c>
       <c r="E368" t="inlineStr">
         <is>
           <t>A</t>
@@ -47493,7 +47593,11 @@
         </is>
       </c>
       <c r="C369" t="inlineStr"/>
-      <c r="D369" t="inlineStr"/>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Omari Nathan Forson</t>
+        </is>
+      </c>
       <c r="E369" t="inlineStr">
         <is>
           <t>A</t>
@@ -47599,7 +47703,11 @@
         </is>
       </c>
       <c r="C370" t="inlineStr"/>
-      <c r="D370" t="inlineStr"/>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Matija Frigan</t>
+        </is>
+      </c>
       <c r="E370" t="inlineStr">
         <is>
           <t>A</t>
@@ -47707,7 +47815,11 @@
         </is>
       </c>
       <c r="C371" s="3" t="inlineStr"/>
-      <c r="D371" s="3" t="inlineStr"/>
+      <c r="D371" s="3" t="inlineStr">
+        <is>
+          <t>Willem Davnis Louis Didier Geubbels</t>
+        </is>
+      </c>
       <c r="E371" s="3" t="inlineStr">
         <is>
           <t>A</t>
@@ -47833,7 +47945,11 @@
         </is>
       </c>
       <c r="C372" t="inlineStr"/>
-      <c r="D372" t="inlineStr"/>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Farès Ghedjemis</t>
+        </is>
+      </c>
       <c r="E372" t="inlineStr">
         <is>
           <t>A</t>
@@ -48051,7 +48167,11 @@
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr"/>
-      <c r="D374" s="2" t="inlineStr"/>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>Gonçalo Matias Ramos</t>
+        </is>
+      </c>
       <c r="E374" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -48163,7 +48283,11 @@
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr"/>
-      <c r="D375" s="2" t="inlineStr"/>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>Nicolás Iván González</t>
+        </is>
+      </c>
       <c r="E375" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -48275,7 +48399,11 @@
         </is>
       </c>
       <c r="C376" t="inlineStr"/>
-      <c r="D376" t="inlineStr"/>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Idrissa Gueye</t>
+        </is>
+      </c>
       <c r="E376" t="inlineStr">
         <is>
           <t>A</t>
@@ -48407,7 +48535,11 @@
         </is>
       </c>
       <c r="C377" t="inlineStr"/>
-      <c r="D377" t="inlineStr"/>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Gustavo Miguel Pereira de Sousa Varela</t>
+        </is>
+      </c>
       <c r="E377" t="inlineStr">
         <is>
           <t>A</t>
@@ -48517,7 +48649,11 @@
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr"/>
-      <c r="D378" s="2" t="inlineStr"/>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>Rasmus Winther Højlund</t>
+        </is>
+      </c>
       <c r="E378" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -48917,7 +49053,11 @@
         </is>
       </c>
       <c r="C381" t="inlineStr"/>
-      <c r="D381" t="inlineStr"/>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Moise Bioty Kean</t>
+        </is>
+      </c>
       <c r="E381" t="inlineStr">
         <is>
           <t>A</t>
@@ -49157,7 +49297,11 @@
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr"/>
-      <c r="D383" s="2" t="inlineStr"/>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>Randal Kolo Muani</t>
+        </is>
+      </c>
       <c r="E383" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -49269,7 +49413,11 @@
         </is>
       </c>
       <c r="C384" t="inlineStr"/>
-      <c r="D384" t="inlineStr"/>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Nikola Krstović</t>
+        </is>
+      </c>
       <c r="E384" t="inlineStr">
         <is>
           <t>A</t>
@@ -49641,7 +49789,11 @@
         </is>
       </c>
       <c r="C387" t="inlineStr"/>
-      <c r="D387" t="inlineStr"/>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Giorgi Kvernadze</t>
+        </is>
+      </c>
       <c r="E387" t="inlineStr">
         <is>
           <t>A</t>
@@ -49751,7 +49903,11 @@
         </is>
       </c>
       <c r="C388" t="inlineStr"/>
-      <c r="D388" t="inlineStr"/>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Noa Noëll Lang</t>
+        </is>
+      </c>
       <c r="E388" t="inlineStr">
         <is>
           <t>A</t>
@@ -49965,7 +50121,11 @@
         </is>
       </c>
       <c r="C390" s="4" t="inlineStr"/>
-      <c r="D390" s="4" t="inlineStr"/>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>Armand Gaëtan Laurienté</t>
+        </is>
+      </c>
       <c r="E390" s="4" t="inlineStr">
         <is>
           <t>A</t>
@@ -50104,8 +50264,16 @@
           <t>Lautaro Martinez</t>
         </is>
       </c>
-      <c r="C391" s="2" t="inlineStr"/>
-      <c r="D391" s="2" t="inlineStr"/>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>el Toro</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>Lautaro Javier Martínez</t>
+        </is>
+      </c>
       <c r="E391" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -50241,7 +50409,11 @@
         </is>
       </c>
       <c r="C392" t="inlineStr"/>
-      <c r="D392" t="inlineStr"/>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Simone Lontani</t>
+        </is>
+      </c>
       <c r="E392" t="inlineStr">
         <is>
           <t>A</t>
@@ -50353,7 +50525,11 @@
         </is>
       </c>
       <c r="C393" t="inlineStr"/>
-      <c r="D393" t="inlineStr"/>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Lorenzo Lucca</t>
+        </is>
+      </c>
       <c r="E393" t="inlineStr">
         <is>
           <t>A</t>
@@ -50461,7 +50637,11 @@
         </is>
       </c>
       <c r="C394" s="4" t="inlineStr"/>
-      <c r="D394" s="4" t="inlineStr"/>
+      <c r="D394" s="4" t="inlineStr">
+        <is>
+          <t>Donyell Malen</t>
+        </is>
+      </c>
       <c r="E394" s="4" t="inlineStr">
         <is>
           <t>A</t>
@@ -50601,7 +50781,11 @@
         </is>
       </c>
       <c r="C395" t="inlineStr"/>
-      <c r="D395" t="inlineStr"/>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Paul Mendy</t>
+        </is>
+      </c>
       <c r="E395" t="inlineStr">
         <is>
           <t>A</t>
@@ -50869,7 +51053,11 @@
         </is>
       </c>
       <c r="C397" t="inlineStr"/>
-      <c r="D397" t="inlineStr"/>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Tijjani Noslin</t>
+        </is>
+      </c>
       <c r="E397" t="inlineStr">
         <is>
           <t>A</t>
@@ -51241,7 +51429,11 @@
         </is>
       </c>
       <c r="C400" t="inlineStr"/>
-      <c r="D400" t="inlineStr"/>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Milutin Osmajić</t>
+        </is>
+      </c>
       <c r="E400" t="inlineStr">
         <is>
           <t>A</t>
@@ -51565,7 +51757,11 @@
         </is>
       </c>
       <c r="C403" t="inlineStr"/>
-      <c r="D403" t="inlineStr"/>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Mateo Pellegrino Casalánguida</t>
+        </is>
+      </c>
       <c r="E403" t="inlineStr">
         <is>
           <t>A</t>
@@ -51697,7 +51893,11 @@
         </is>
       </c>
       <c r="C404" t="inlineStr"/>
-      <c r="D404" t="inlineStr"/>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Roberto Piccoli</t>
+        </is>
+      </c>
       <c r="E404" t="inlineStr">
         <is>
           <t>A</t>
@@ -51969,7 +52169,11 @@
         </is>
       </c>
       <c r="C406" t="inlineStr"/>
-      <c r="D406" t="inlineStr"/>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Antonio Raimondo</t>
+        </is>
+      </c>
       <c r="E406" t="inlineStr">
         <is>
           <t>A</t>
@@ -52079,7 +52283,11 @@
         </is>
       </c>
       <c r="C407" t="inlineStr"/>
-      <c r="D407" t="inlineStr"/>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Giacomo Raspadori</t>
+        </is>
+      </c>
       <c r="E407" t="inlineStr">
         <is>
           <t>A</t>
@@ -52211,7 +52419,11 @@
         </is>
       </c>
       <c r="C408" t="inlineStr"/>
-      <c r="D408" t="inlineStr"/>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Jay Steven Robinson</t>
+        </is>
+      </c>
       <c r="E408" t="inlineStr">
         <is>
           <t>A</t>
@@ -52317,7 +52529,11 @@
         </is>
       </c>
       <c r="C409" t="inlineStr"/>
-      <c r="D409" t="inlineStr"/>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>José David Romero</t>
+        </is>
+      </c>
       <c r="E409" t="inlineStr">
         <is>
           <t>A</t>
@@ -52429,7 +52645,11 @@
         </is>
       </c>
       <c r="C410" t="inlineStr"/>
-      <c r="D410" t="inlineStr"/>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Jonathan David Henry Rowe</t>
+        </is>
+      </c>
       <c r="E410" t="inlineStr">
         <is>
           <t>A</t>
@@ -52561,7 +52781,11 @@
         </is>
       </c>
       <c r="C411" t="inlineStr"/>
-      <c r="D411" t="inlineStr"/>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Gianluca Scamacca</t>
+        </is>
+      </c>
       <c r="E411" t="inlineStr">
         <is>
           <t>A</t>
@@ -52833,7 +53057,11 @@
         </is>
       </c>
       <c r="C413" s="2" t="inlineStr"/>
-      <c r="D413" s="2" t="inlineStr"/>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>Matías Soulé Malvano</t>
+        </is>
+      </c>
       <c r="E413" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -52969,7 +53197,11 @@
         </is>
       </c>
       <c r="C414" t="inlineStr"/>
-      <c r="D414" t="inlineStr"/>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Nikola Štulić</t>
+        </is>
+      </c>
       <c r="E414" t="inlineStr">
         <is>
           <t>A</t>
@@ -53105,7 +53337,11 @@
         </is>
       </c>
       <c r="C415" t="inlineStr"/>
-      <c r="D415" t="inlineStr"/>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Alessandro Sugamele</t>
+        </is>
+      </c>
       <c r="E415" t="inlineStr">
         <is>
           <t>A</t>
@@ -53213,7 +53449,11 @@
         </is>
       </c>
       <c r="C416" s="2" t="inlineStr"/>
-      <c r="D416" s="2" t="inlineStr"/>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>Marcus Lilian Thuram-Ulien</t>
+        </is>
+      </c>
       <c r="E416" s="2" t="inlineStr">
         <is>
           <t>A</t>
@@ -53349,7 +53589,11 @@
         </is>
       </c>
       <c r="C417" t="inlineStr"/>
-      <c r="D417" t="inlineStr"/>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>El Bilal Touré</t>
+        </is>
+      </c>
       <c r="E417" t="inlineStr">
         <is>
           <t>A</t>
@@ -53457,7 +53701,11 @@
         </is>
       </c>
       <c r="C418" t="inlineStr"/>
-      <c r="D418" t="inlineStr"/>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Vítor Manuel Carvalho Oliveira</t>
+        </is>
+      </c>
       <c r="E418" t="inlineStr">
         <is>
           <t>A</t>
@@ -53697,7 +53945,11 @@
         </is>
       </c>
       <c r="C420" t="inlineStr"/>
-      <c r="D420" t="inlineStr"/>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>John Yeboah Zamora</t>
+        </is>
+      </c>
       <c r="E420" t="inlineStr">
         <is>
           <t>A</t>
@@ -53811,7 +54063,11 @@
         </is>
       </c>
       <c r="C421" s="3" t="inlineStr"/>
-      <c r="D421" s="3" t="inlineStr"/>
+      <c r="D421" s="3" t="inlineStr">
+        <is>
+          <t>Kenan Yıldız</t>
+        </is>
+      </c>
       <c r="E421" s="3" t="inlineStr">
         <is>
           <t>A</t>
@@ -54087,7 +54343,11 @@
         </is>
       </c>
       <c r="C423" t="inlineStr"/>
-      <c r="D423" t="inlineStr"/>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Oscar Exequiel Zeballos</t>
+        </is>
+      </c>
       <c r="E423" t="inlineStr">
         <is>
           <t>A</t>
@@ -62263,7 +62523,11 @@
           <t>Lautaro Martinez</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>el Toro</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Inter</t>
@@ -66500,7 +66764,11 @@
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Armand Gaëtan Laurienté</t>
+        </is>
+      </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>A</t>
@@ -66643,7 +66911,11 @@
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Donyell Malen</t>
+        </is>
+      </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
           <t>A</t>

</xml_diff>